<commit_message>
Update renxiao dashboard and publish snapshot
</commit_message>
<xml_diff>
--- a/data/uploads/renxiaomubiao_demo.xlsx
+++ b/data/uploads/renxiaomubiao_demo.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="26860" windowHeight="11140"/>
+    <workbookView windowWidth="26860" windowHeight="11740"/>
   </bookViews>
   <sheets>
     <sheet name="sheet" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="8">
   <si>
     <t>日期</t>
   </si>
@@ -60,12 +60,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="[$-409]yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="177" formatCode="0.0_ "/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -694,7 +695,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -708,6 +709,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
@@ -1099,7 +1103,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:T232"/>
+  <dimension ref="A1:T277"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="12.5" customWidth="1"/>
@@ -1953,1177 +1957,2658 @@
       <c r="E65" s="5"/>
     </row>
     <row r="66" spans="1:5">
-      <c r="A66" s="5"/>
-      <c r="B66" s="3"/>
-      <c r="C66" s="4"/>
+      <c r="A66" s="2">
+        <v>46266</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C66" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D66" s="5"/>
       <c r="E66" s="5"/>
     </row>
     <row r="67" spans="1:5">
-      <c r="A67" s="5"/>
-      <c r="B67" s="3"/>
-      <c r="C67" s="4"/>
+      <c r="A67" s="2">
+        <v>46267</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C67" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D67" s="5"/>
       <c r="E67" s="5"/>
     </row>
     <row r="68" spans="1:5">
-      <c r="A68" s="5"/>
-      <c r="B68" s="3"/>
-      <c r="C68" s="4"/>
+      <c r="A68" s="2">
+        <v>46268</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C68" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D68" s="5"/>
       <c r="E68" s="5"/>
     </row>
     <row r="69" spans="1:5">
-      <c r="A69" s="5"/>
-      <c r="B69" s="3"/>
-      <c r="C69" s="4"/>
+      <c r="A69" s="2">
+        <v>46269</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C69" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D69" s="5"/>
       <c r="E69" s="5"/>
     </row>
     <row r="70" spans="1:5">
-      <c r="A70" s="5"/>
-      <c r="B70" s="3"/>
-      <c r="C70" s="4"/>
+      <c r="A70" s="2">
+        <v>46270</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C70" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D70" s="5"/>
       <c r="E70" s="5"/>
     </row>
     <row r="71" spans="1:5">
-      <c r="A71" s="5"/>
-      <c r="B71" s="3"/>
-      <c r="C71" s="4"/>
+      <c r="A71" s="2">
+        <v>46271</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C71" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D71" s="5"/>
       <c r="E71" s="5"/>
     </row>
     <row r="72" spans="1:5">
-      <c r="A72" s="5"/>
-      <c r="B72" s="3"/>
-      <c r="C72" s="4"/>
+      <c r="A72" s="2">
+        <v>46272</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C72" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D72" s="5"/>
       <c r="E72" s="5"/>
     </row>
     <row r="73" spans="1:5">
-      <c r="A73" s="5"/>
-      <c r="B73" s="3"/>
-      <c r="C73" s="4"/>
+      <c r="A73" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C73" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D73" s="5"/>
       <c r="E73" s="5"/>
     </row>
     <row r="74" spans="1:5">
-      <c r="A74" s="5"/>
-      <c r="B74" s="3"/>
-      <c r="C74" s="4"/>
+      <c r="A74" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B74" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C74" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D74" s="5"/>
       <c r="E74" s="5"/>
     </row>
     <row r="75" spans="1:5">
-      <c r="A75" s="5"/>
-      <c r="B75" s="3"/>
-      <c r="C75" s="4"/>
+      <c r="A75" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B75" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C75" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D75" s="5"/>
       <c r="E75" s="5"/>
     </row>
     <row r="76" spans="1:5">
-      <c r="A76" s="5"/>
-      <c r="B76" s="3"/>
-      <c r="C76" s="4"/>
+      <c r="A76" s="2">
+        <v>46276</v>
+      </c>
+      <c r="B76" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C76" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D76" s="5"/>
       <c r="E76" s="5"/>
     </row>
     <row r="77" spans="1:5">
-      <c r="A77" s="5"/>
-      <c r="B77" s="3"/>
-      <c r="C77" s="4"/>
+      <c r="A77" s="2">
+        <v>46277</v>
+      </c>
+      <c r="B77" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C77" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D77" s="5"/>
       <c r="E77" s="5"/>
     </row>
     <row r="78" spans="1:5">
-      <c r="A78" s="5"/>
-      <c r="B78" s="3"/>
-      <c r="C78" s="4"/>
+      <c r="A78" s="2">
+        <v>46278</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C78" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D78" s="5"/>
       <c r="E78" s="5"/>
     </row>
     <row r="79" spans="1:5">
-      <c r="A79" s="5"/>
-      <c r="B79" s="3"/>
-      <c r="C79" s="4"/>
+      <c r="A79" s="2">
+        <v>46279</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C79" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D79" s="5"/>
       <c r="E79" s="5"/>
     </row>
     <row r="80" spans="1:5">
-      <c r="A80" s="5"/>
-      <c r="B80" s="3"/>
-      <c r="C80" s="4"/>
+      <c r="A80" s="2">
+        <v>46280</v>
+      </c>
+      <c r="B80" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C80" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D80" s="5"/>
       <c r="E80" s="5"/>
     </row>
     <row r="81" spans="1:5">
-      <c r="A81" s="5"/>
-      <c r="B81" s="3"/>
-      <c r="C81" s="4"/>
+      <c r="A81" s="2">
+        <v>46281</v>
+      </c>
+      <c r="B81" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C81" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D81" s="5"/>
       <c r="E81" s="5"/>
     </row>
     <row r="82" spans="1:5">
-      <c r="A82" s="5"/>
-      <c r="B82" s="3"/>
-      <c r="C82" s="4"/>
+      <c r="A82" s="2">
+        <v>46282</v>
+      </c>
+      <c r="B82" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C82" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D82" s="5"/>
       <c r="E82" s="5"/>
     </row>
     <row r="83" spans="1:5">
-      <c r="A83" s="5"/>
-      <c r="B83" s="3"/>
-      <c r="C83" s="4"/>
+      <c r="A83" s="2">
+        <v>46283</v>
+      </c>
+      <c r="B83" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C83" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D83" s="5"/>
       <c r="E83" s="5"/>
     </row>
     <row r="84" spans="1:5">
-      <c r="A84" s="5"/>
-      <c r="B84" s="3"/>
-      <c r="C84" s="4"/>
+      <c r="A84" s="2">
+        <v>46284</v>
+      </c>
+      <c r="B84" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C84" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D84" s="5"/>
       <c r="E84" s="5"/>
     </row>
     <row r="85" spans="1:5">
-      <c r="A85" s="5"/>
-      <c r="B85" s="3"/>
-      <c r="C85" s="4"/>
+      <c r="A85" s="2">
+        <v>46285</v>
+      </c>
+      <c r="B85" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C85" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D85" s="5"/>
       <c r="E85" s="5"/>
     </row>
     <row r="86" spans="1:5">
-      <c r="A86" s="5"/>
-      <c r="B86" s="3"/>
-      <c r="C86" s="4"/>
+      <c r="A86" s="2">
+        <v>46286</v>
+      </c>
+      <c r="B86" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C86" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D86" s="5"/>
       <c r="E86" s="5"/>
     </row>
     <row r="87" spans="1:5">
-      <c r="A87" s="5"/>
-      <c r="B87" s="3"/>
-      <c r="C87" s="4"/>
+      <c r="A87" s="2">
+        <v>46287</v>
+      </c>
+      <c r="B87" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C87" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D87" s="5"/>
       <c r="E87" s="5"/>
     </row>
     <row r="88" spans="1:5">
-      <c r="A88" s="5"/>
-      <c r="B88" s="3"/>
-      <c r="C88" s="4"/>
+      <c r="A88" s="2">
+        <v>46288</v>
+      </c>
+      <c r="B88" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C88" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D88" s="5"/>
       <c r="E88" s="5"/>
     </row>
     <row r="89" spans="1:5">
-      <c r="A89" s="5"/>
-      <c r="B89" s="3"/>
-      <c r="C89" s="4"/>
+      <c r="A89" s="2">
+        <v>46289</v>
+      </c>
+      <c r="B89" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C89" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D89" s="5"/>
       <c r="E89" s="5"/>
     </row>
     <row r="90" spans="1:5">
-      <c r="A90" s="5"/>
-      <c r="B90" s="3"/>
-      <c r="C90" s="4"/>
+      <c r="A90" s="2">
+        <v>46290</v>
+      </c>
+      <c r="B90" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C90" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D90" s="5"/>
       <c r="E90" s="5"/>
     </row>
     <row r="91" spans="1:5">
-      <c r="A91" s="5"/>
-      <c r="B91" s="3"/>
-      <c r="C91" s="4"/>
+      <c r="A91" s="2">
+        <v>46291</v>
+      </c>
+      <c r="B91" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C91" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D91" s="5"/>
       <c r="E91" s="5"/>
     </row>
     <row r="92" spans="1:5">
-      <c r="A92" s="5"/>
-      <c r="B92" s="3"/>
-      <c r="C92" s="4"/>
+      <c r="A92" s="2">
+        <v>46292</v>
+      </c>
+      <c r="B92" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C92" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D92" s="5"/>
       <c r="E92" s="5"/>
     </row>
     <row r="93" spans="1:5">
-      <c r="A93" s="5"/>
-      <c r="B93" s="3"/>
-      <c r="C93" s="4"/>
+      <c r="A93" s="2">
+        <v>46293</v>
+      </c>
+      <c r="B93" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C93" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D93" s="5"/>
       <c r="E93" s="5"/>
     </row>
     <row r="94" spans="1:5">
-      <c r="A94" s="5"/>
-      <c r="B94" s="3"/>
-      <c r="C94" s="4"/>
+      <c r="A94" s="2">
+        <v>46294</v>
+      </c>
+      <c r="B94" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C94" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D94" s="5"/>
       <c r="E94" s="5"/>
     </row>
     <row r="95" spans="1:5">
-      <c r="A95" s="5"/>
-      <c r="B95" s="3"/>
-      <c r="C95" s="4"/>
+      <c r="A95" s="2">
+        <v>46295</v>
+      </c>
+      <c r="B95" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C95" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D95" s="5"/>
       <c r="E95" s="5"/>
     </row>
     <row r="96" spans="1:5">
-      <c r="A96" s="5"/>
-      <c r="B96" s="3"/>
-      <c r="C96" s="4"/>
+      <c r="A96" s="2">
+        <v>46266</v>
+      </c>
+      <c r="B96" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C96" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D96" s="5"/>
       <c r="E96" s="5"/>
     </row>
     <row r="97" spans="1:5">
-      <c r="A97" s="5"/>
-      <c r="B97" s="3"/>
-      <c r="C97" s="4"/>
+      <c r="A97" s="2">
+        <v>46267</v>
+      </c>
+      <c r="B97" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C97" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D97" s="5"/>
       <c r="E97" s="5"/>
     </row>
     <row r="98" spans="1:5">
-      <c r="A98" s="5"/>
-      <c r="B98" s="3"/>
-      <c r="C98" s="4"/>
+      <c r="A98" s="2">
+        <v>46268</v>
+      </c>
+      <c r="B98" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C98" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D98" s="5"/>
       <c r="E98" s="5"/>
     </row>
     <row r="99" spans="1:5">
-      <c r="A99" s="5"/>
-      <c r="B99" s="3"/>
-      <c r="C99" s="4"/>
+      <c r="A99" s="2">
+        <v>46269</v>
+      </c>
+      <c r="B99" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C99" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D99" s="5"/>
       <c r="E99" s="5"/>
     </row>
     <row r="100" spans="1:5">
-      <c r="A100" s="5"/>
-      <c r="B100" s="3"/>
-      <c r="C100" s="4"/>
+      <c r="A100" s="2">
+        <v>46270</v>
+      </c>
+      <c r="B100" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C100" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D100" s="5"/>
       <c r="E100" s="5"/>
     </row>
     <row r="101" spans="1:5">
-      <c r="A101" s="5"/>
-      <c r="B101" s="3"/>
-      <c r="C101" s="4"/>
+      <c r="A101" s="2">
+        <v>46271</v>
+      </c>
+      <c r="B101" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C101" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D101" s="5"/>
       <c r="E101" s="5"/>
     </row>
     <row r="102" spans="1:5">
-      <c r="A102" s="5"/>
-      <c r="B102" s="3"/>
-      <c r="C102" s="4"/>
+      <c r="A102" s="2">
+        <v>46272</v>
+      </c>
+      <c r="B102" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C102" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D102" s="5"/>
       <c r="E102" s="5"/>
     </row>
     <row r="103" spans="1:5">
-      <c r="A103" s="5"/>
-      <c r="B103" s="3"/>
-      <c r="C103" s="4"/>
+      <c r="A103" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B103" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C103" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D103" s="5"/>
       <c r="E103" s="5"/>
     </row>
     <row r="104" spans="1:5">
-      <c r="A104" s="5"/>
-      <c r="B104" s="3"/>
-      <c r="C104" s="4"/>
+      <c r="A104" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B104" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C104" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D104" s="5"/>
       <c r="E104" s="5"/>
     </row>
     <row r="105" spans="1:5">
-      <c r="A105" s="5"/>
-      <c r="B105" s="3"/>
-      <c r="C105" s="4"/>
+      <c r="A105" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B105" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C105" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D105" s="5"/>
       <c r="E105" s="5"/>
     </row>
     <row r="106" spans="1:5">
-      <c r="A106" s="5"/>
-      <c r="B106" s="3"/>
-      <c r="C106" s="4"/>
+      <c r="A106" s="2">
+        <v>46276</v>
+      </c>
+      <c r="B106" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C106" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D106" s="5"/>
       <c r="E106" s="5"/>
     </row>
     <row r="107" spans="1:5">
-      <c r="A107" s="5"/>
-      <c r="B107" s="3"/>
-      <c r="C107" s="4"/>
+      <c r="A107" s="2">
+        <v>46277</v>
+      </c>
+      <c r="B107" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C107" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D107" s="5"/>
       <c r="E107" s="5"/>
     </row>
     <row r="108" spans="1:5">
-      <c r="A108" s="5"/>
-      <c r="B108" s="3"/>
-      <c r="C108" s="4"/>
+      <c r="A108" s="2">
+        <v>46278</v>
+      </c>
+      <c r="B108" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C108" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D108" s="5"/>
       <c r="E108" s="5"/>
     </row>
     <row r="109" spans="1:5">
-      <c r="A109" s="5"/>
-      <c r="B109" s="3"/>
-      <c r="C109" s="4"/>
+      <c r="A109" s="2">
+        <v>46279</v>
+      </c>
+      <c r="B109" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C109" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D109" s="5"/>
       <c r="E109" s="5"/>
     </row>
     <row r="110" spans="1:5">
-      <c r="A110" s="5"/>
-      <c r="B110" s="3"/>
-      <c r="C110" s="4"/>
+      <c r="A110" s="2">
+        <v>46280</v>
+      </c>
+      <c r="B110" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C110" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D110" s="5"/>
       <c r="E110" s="5"/>
     </row>
     <row r="111" spans="1:5">
-      <c r="A111" s="5"/>
-      <c r="B111" s="3"/>
-      <c r="C111" s="4"/>
+      <c r="A111" s="2">
+        <v>46281</v>
+      </c>
+      <c r="B111" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C111" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D111" s="5"/>
       <c r="E111" s="5"/>
     </row>
     <row r="112" spans="1:5">
-      <c r="A112" s="5"/>
-      <c r="B112" s="3"/>
-      <c r="C112" s="4"/>
+      <c r="A112" s="2">
+        <v>46282</v>
+      </c>
+      <c r="B112" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C112" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D112" s="5"/>
       <c r="E112" s="5"/>
     </row>
     <row r="113" spans="1:5">
-      <c r="A113" s="5"/>
-      <c r="B113" s="3"/>
-      <c r="C113" s="4"/>
+      <c r="A113" s="2">
+        <v>46283</v>
+      </c>
+      <c r="B113" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C113" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D113" s="5"/>
       <c r="E113" s="5"/>
     </row>
     <row r="114" spans="1:5">
-      <c r="A114" s="5"/>
-      <c r="B114" s="3"/>
-      <c r="C114" s="4"/>
+      <c r="A114" s="2">
+        <v>46284</v>
+      </c>
+      <c r="B114" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C114" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D114" s="5"/>
       <c r="E114" s="5"/>
     </row>
     <row r="115" spans="1:5">
-      <c r="A115" s="5"/>
-      <c r="B115" s="3"/>
-      <c r="C115" s="4"/>
+      <c r="A115" s="2">
+        <v>46285</v>
+      </c>
+      <c r="B115" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C115" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D115" s="5"/>
       <c r="E115" s="5"/>
     </row>
     <row r="116" spans="1:5">
-      <c r="A116" s="5"/>
-      <c r="B116" s="3"/>
-      <c r="C116" s="4"/>
+      <c r="A116" s="2">
+        <v>46286</v>
+      </c>
+      <c r="B116" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C116" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D116" s="5"/>
       <c r="E116" s="5"/>
     </row>
     <row r="117" spans="1:5">
-      <c r="A117" s="5"/>
-      <c r="B117" s="3"/>
-      <c r="C117" s="4"/>
+      <c r="A117" s="2">
+        <v>46287</v>
+      </c>
+      <c r="B117" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C117" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D117" s="5"/>
       <c r="E117" s="5"/>
     </row>
     <row r="118" spans="1:5">
-      <c r="A118" s="5"/>
-      <c r="B118" s="3"/>
-      <c r="C118" s="4"/>
+      <c r="A118" s="2">
+        <v>46288</v>
+      </c>
+      <c r="B118" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C118" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D118" s="5"/>
       <c r="E118" s="5"/>
     </row>
     <row r="119" spans="1:5">
-      <c r="A119" s="5"/>
-      <c r="B119" s="3"/>
-      <c r="C119" s="4"/>
+      <c r="A119" s="2">
+        <v>46289</v>
+      </c>
+      <c r="B119" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C119" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D119" s="5"/>
       <c r="E119" s="5"/>
     </row>
     <row r="120" spans="1:5">
-      <c r="A120" s="5"/>
-      <c r="B120" s="3"/>
-      <c r="C120" s="4"/>
+      <c r="A120" s="2">
+        <v>46290</v>
+      </c>
+      <c r="B120" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C120" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D120" s="5"/>
       <c r="E120" s="5"/>
     </row>
     <row r="121" spans="1:5">
-      <c r="A121" s="5"/>
-      <c r="B121" s="3"/>
-      <c r="C121" s="4"/>
+      <c r="A121" s="2">
+        <v>46291</v>
+      </c>
+      <c r="B121" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C121" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D121" s="5"/>
       <c r="E121" s="5"/>
     </row>
     <row r="122" spans="1:5">
-      <c r="A122" s="5"/>
-      <c r="B122" s="3"/>
-      <c r="C122" s="4"/>
+      <c r="A122" s="2">
+        <v>46292</v>
+      </c>
+      <c r="B122" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C122" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D122" s="5"/>
       <c r="E122" s="5"/>
     </row>
     <row r="123" spans="1:5">
-      <c r="A123" s="5"/>
-      <c r="B123" s="3"/>
-      <c r="C123" s="4"/>
+      <c r="A123" s="2">
+        <v>46293</v>
+      </c>
+      <c r="B123" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C123" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D123" s="5"/>
       <c r="E123" s="5"/>
     </row>
     <row r="124" spans="1:5">
-      <c r="A124" s="5"/>
-      <c r="B124" s="3"/>
-      <c r="C124" s="4"/>
+      <c r="A124" s="2">
+        <v>46294</v>
+      </c>
+      <c r="B124" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C124" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D124" s="5"/>
       <c r="E124" s="5"/>
     </row>
     <row r="125" spans="1:5">
-      <c r="A125" s="5"/>
-      <c r="B125" s="3"/>
-      <c r="C125" s="4"/>
+      <c r="A125" s="2">
+        <v>46295</v>
+      </c>
+      <c r="B125" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C125" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D125" s="5"/>
       <c r="E125" s="5"/>
     </row>
     <row r="126" spans="1:5">
-      <c r="A126" s="5"/>
-      <c r="B126" s="3"/>
-      <c r="C126" s="4"/>
+      <c r="A126" s="2">
+        <v>46266</v>
+      </c>
+      <c r="B126" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C126" s="9">
+        <v>6</v>
+      </c>
       <c r="D126" s="5"/>
       <c r="E126" s="5"/>
     </row>
     <row r="127" spans="1:5">
-      <c r="A127" s="5"/>
-      <c r="B127" s="3"/>
-      <c r="C127" s="4"/>
+      <c r="A127" s="2">
+        <v>46267</v>
+      </c>
+      <c r="B127" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C127" s="9">
+        <v>6</v>
+      </c>
       <c r="D127" s="5"/>
       <c r="E127" s="5"/>
     </row>
     <row r="128" spans="1:5">
-      <c r="A128" s="5"/>
-      <c r="B128" s="3"/>
-      <c r="C128" s="4"/>
+      <c r="A128" s="2">
+        <v>46268</v>
+      </c>
+      <c r="B128" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C128" s="9">
+        <v>6</v>
+      </c>
       <c r="D128" s="5"/>
       <c r="E128" s="5"/>
     </row>
     <row r="129" spans="1:5">
-      <c r="A129" s="5"/>
-      <c r="B129" s="3"/>
-      <c r="C129" s="4"/>
+      <c r="A129" s="2">
+        <v>46269</v>
+      </c>
+      <c r="B129" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C129" s="9">
+        <v>6</v>
+      </c>
       <c r="D129" s="5"/>
       <c r="E129" s="5"/>
     </row>
     <row r="130" spans="1:5">
-      <c r="A130" s="5"/>
-      <c r="B130" s="3"/>
-      <c r="C130" s="4"/>
+      <c r="A130" s="2">
+        <v>46270</v>
+      </c>
+      <c r="B130" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C130" s="9">
+        <v>6</v>
+      </c>
       <c r="D130" s="5"/>
       <c r="E130" s="5"/>
     </row>
     <row r="131" spans="1:5">
-      <c r="A131" s="5"/>
-      <c r="B131" s="3"/>
-      <c r="C131" s="4"/>
+      <c r="A131" s="2">
+        <v>46271</v>
+      </c>
+      <c r="B131" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C131" s="9">
+        <v>6</v>
+      </c>
       <c r="D131" s="5"/>
       <c r="E131" s="5"/>
     </row>
     <row r="132" spans="1:5">
-      <c r="A132" s="5"/>
-      <c r="B132" s="3"/>
-      <c r="C132" s="4"/>
+      <c r="A132" s="2">
+        <v>46272</v>
+      </c>
+      <c r="B132" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C132" s="9">
+        <v>6</v>
+      </c>
       <c r="D132" s="5"/>
       <c r="E132" s="5"/>
     </row>
     <row r="133" spans="1:5">
-      <c r="A133" s="5"/>
-      <c r="B133" s="3"/>
-      <c r="C133" s="4"/>
+      <c r="A133" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B133" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C133" s="9">
+        <v>6</v>
+      </c>
       <c r="D133" s="5"/>
       <c r="E133" s="5"/>
     </row>
     <row r="134" spans="1:5">
-      <c r="A134" s="5"/>
-      <c r="B134" s="3"/>
-      <c r="C134" s="4"/>
+      <c r="A134" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B134" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C134" s="9">
+        <v>6</v>
+      </c>
       <c r="D134" s="5"/>
       <c r="E134" s="5"/>
     </row>
     <row r="135" spans="1:5">
-      <c r="A135" s="5"/>
-      <c r="B135" s="3"/>
-      <c r="C135" s="4"/>
+      <c r="A135" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B135" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C135" s="9">
+        <v>6</v>
+      </c>
       <c r="D135" s="5"/>
       <c r="E135" s="5"/>
     </row>
     <row r="136" spans="1:5">
-      <c r="A136" s="5"/>
-      <c r="B136" s="3"/>
-      <c r="C136" s="4"/>
+      <c r="A136" s="2">
+        <v>46276</v>
+      </c>
+      <c r="B136" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C136" s="9">
+        <v>6</v>
+      </c>
       <c r="D136" s="5"/>
       <c r="E136" s="5"/>
     </row>
     <row r="137" spans="1:5">
-      <c r="A137" s="5"/>
-      <c r="B137" s="3"/>
-      <c r="C137" s="4"/>
+      <c r="A137" s="2">
+        <v>46277</v>
+      </c>
+      <c r="B137" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C137" s="9">
+        <v>6</v>
+      </c>
       <c r="D137" s="5"/>
       <c r="E137" s="5"/>
     </row>
     <row r="138" spans="1:5">
-      <c r="A138" s="5"/>
-      <c r="B138" s="3"/>
-      <c r="C138" s="4"/>
+      <c r="A138" s="2">
+        <v>46278</v>
+      </c>
+      <c r="B138" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C138" s="9">
+        <v>6</v>
+      </c>
       <c r="D138" s="5"/>
       <c r="E138" s="5"/>
     </row>
     <row r="139" spans="1:5">
-      <c r="A139" s="5"/>
-      <c r="B139" s="3"/>
-      <c r="C139" s="4"/>
+      <c r="A139" s="2">
+        <v>46279</v>
+      </c>
+      <c r="B139" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C139" s="9">
+        <v>6</v>
+      </c>
       <c r="D139" s="5"/>
       <c r="E139" s="5"/>
     </row>
     <row r="140" spans="1:5">
-      <c r="A140" s="5"/>
-      <c r="B140" s="3"/>
-      <c r="C140" s="4"/>
+      <c r="A140" s="2">
+        <v>46280</v>
+      </c>
+      <c r="B140" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C140" s="9">
+        <v>6</v>
+      </c>
       <c r="D140" s="5"/>
       <c r="E140" s="5"/>
     </row>
     <row r="141" spans="1:5">
-      <c r="A141" s="5"/>
-      <c r="B141" s="3"/>
-      <c r="C141" s="4"/>
+      <c r="A141" s="2">
+        <v>46281</v>
+      </c>
+      <c r="B141" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C141" s="9">
+        <v>6</v>
+      </c>
       <c r="D141" s="5"/>
       <c r="E141" s="5"/>
     </row>
     <row r="142" spans="1:5">
-      <c r="A142" s="5"/>
-      <c r="B142" s="3"/>
-      <c r="C142" s="4"/>
+      <c r="A142" s="2">
+        <v>46282</v>
+      </c>
+      <c r="B142" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C142" s="9">
+        <v>6</v>
+      </c>
       <c r="D142" s="5"/>
       <c r="E142" s="5"/>
     </row>
     <row r="143" spans="1:5">
-      <c r="A143" s="5"/>
-      <c r="B143" s="3"/>
-      <c r="C143" s="4"/>
+      <c r="A143" s="2">
+        <v>46283</v>
+      </c>
+      <c r="B143" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C143" s="9">
+        <v>6</v>
+      </c>
       <c r="D143" s="5"/>
       <c r="E143" s="5"/>
     </row>
     <row r="144" spans="1:5">
-      <c r="A144" s="5"/>
-      <c r="B144" s="3"/>
-      <c r="C144" s="4"/>
+      <c r="A144" s="2">
+        <v>46284</v>
+      </c>
+      <c r="B144" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C144" s="9">
+        <v>6</v>
+      </c>
       <c r="D144" s="5"/>
       <c r="E144" s="5"/>
     </row>
     <row r="145" spans="1:5">
-      <c r="A145" s="5"/>
-      <c r="B145" s="3"/>
-      <c r="C145" s="4"/>
+      <c r="A145" s="2">
+        <v>46285</v>
+      </c>
+      <c r="B145" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C145" s="9">
+        <v>6</v>
+      </c>
       <c r="D145" s="5"/>
       <c r="E145" s="5"/>
     </row>
     <row r="146" spans="1:5">
-      <c r="A146" s="5"/>
-      <c r="B146" s="3"/>
-      <c r="C146" s="4"/>
+      <c r="A146" s="2">
+        <v>46286</v>
+      </c>
+      <c r="B146" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C146" s="9">
+        <v>6</v>
+      </c>
       <c r="D146" s="5"/>
       <c r="E146" s="5"/>
     </row>
     <row r="147" spans="1:5">
-      <c r="A147" s="5"/>
-      <c r="B147" s="3"/>
-      <c r="C147" s="4"/>
+      <c r="A147" s="2">
+        <v>46287</v>
+      </c>
+      <c r="B147" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C147" s="9">
+        <v>6</v>
+      </c>
       <c r="D147" s="5"/>
       <c r="E147" s="5"/>
     </row>
     <row r="148" spans="1:5">
-      <c r="A148" s="5"/>
-      <c r="B148" s="3"/>
-      <c r="C148" s="4"/>
+      <c r="A148" s="2">
+        <v>46288</v>
+      </c>
+      <c r="B148" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C148" s="9">
+        <v>6</v>
+      </c>
       <c r="D148" s="5"/>
       <c r="E148" s="5"/>
     </row>
     <row r="149" spans="1:5">
-      <c r="A149" s="5"/>
-      <c r="B149" s="3"/>
-      <c r="C149" s="4"/>
+      <c r="A149" s="2">
+        <v>46289</v>
+      </c>
+      <c r="B149" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C149" s="9">
+        <v>6</v>
+      </c>
       <c r="D149" s="5"/>
       <c r="E149" s="5"/>
     </row>
     <row r="150" spans="1:5">
-      <c r="A150" s="5"/>
-      <c r="B150" s="3"/>
-      <c r="C150" s="4"/>
+      <c r="A150" s="2">
+        <v>46290</v>
+      </c>
+      <c r="B150" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C150" s="9">
+        <v>6</v>
+      </c>
       <c r="D150" s="5"/>
       <c r="E150" s="5"/>
     </row>
     <row r="151" spans="1:5">
-      <c r="A151" s="5"/>
-      <c r="B151" s="3"/>
-      <c r="C151" s="4"/>
+      <c r="A151" s="2">
+        <v>46291</v>
+      </c>
+      <c r="B151" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C151" s="9">
+        <v>6</v>
+      </c>
       <c r="D151" s="5"/>
       <c r="E151" s="5"/>
     </row>
     <row r="152" spans="1:5">
-      <c r="A152" s="5"/>
-      <c r="B152" s="3"/>
-      <c r="C152" s="4"/>
+      <c r="A152" s="2">
+        <v>46292</v>
+      </c>
+      <c r="B152" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C152" s="9">
+        <v>6</v>
+      </c>
       <c r="D152" s="5"/>
       <c r="E152" s="5"/>
     </row>
     <row r="153" spans="1:5">
-      <c r="A153" s="5"/>
-      <c r="B153" s="3"/>
-      <c r="C153" s="4"/>
+      <c r="A153" s="2">
+        <v>46293</v>
+      </c>
+      <c r="B153" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C153" s="9">
+        <v>6</v>
+      </c>
       <c r="D153" s="5"/>
       <c r="E153" s="5"/>
     </row>
     <row r="154" spans="1:5">
-      <c r="A154" s="5"/>
-      <c r="B154" s="3"/>
-      <c r="C154" s="4"/>
+      <c r="A154" s="2">
+        <v>46294</v>
+      </c>
+      <c r="B154" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C154" s="9">
+        <v>6</v>
+      </c>
       <c r="D154" s="5"/>
       <c r="E154" s="5"/>
     </row>
     <row r="155" spans="1:5">
-      <c r="A155" s="5"/>
-      <c r="B155" s="3"/>
-      <c r="C155" s="4"/>
+      <c r="A155" s="2">
+        <v>46295</v>
+      </c>
+      <c r="B155" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C155" s="9">
+        <v>6</v>
+      </c>
       <c r="D155" s="5"/>
       <c r="E155" s="5"/>
     </row>
     <row r="156" spans="1:5">
-      <c r="A156" s="5"/>
-      <c r="B156" s="3"/>
-      <c r="C156" s="4"/>
+      <c r="A156" s="2">
+        <v>46266</v>
+      </c>
+      <c r="B156" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C156" s="9">
+        <v>6</v>
+      </c>
       <c r="D156" s="5"/>
       <c r="E156" s="5"/>
     </row>
     <row r="157" spans="1:5">
-      <c r="A157" s="5"/>
-      <c r="B157" s="3"/>
-      <c r="C157" s="4"/>
+      <c r="A157" s="2">
+        <v>46267</v>
+      </c>
+      <c r="B157" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C157" s="9">
+        <v>6</v>
+      </c>
       <c r="D157" s="5"/>
       <c r="E157" s="5"/>
     </row>
     <row r="158" spans="1:5">
-      <c r="A158" s="5"/>
-      <c r="B158" s="3"/>
-      <c r="C158" s="4"/>
+      <c r="A158" s="2">
+        <v>46268</v>
+      </c>
+      <c r="B158" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C158" s="9">
+        <v>6</v>
+      </c>
       <c r="D158" s="5"/>
       <c r="E158" s="5"/>
     </row>
     <row r="159" spans="1:5">
-      <c r="A159" s="5"/>
-      <c r="B159" s="3"/>
-      <c r="C159" s="4"/>
+      <c r="A159" s="2">
+        <v>46269</v>
+      </c>
+      <c r="B159" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C159" s="9">
+        <v>6</v>
+      </c>
       <c r="D159" s="5"/>
       <c r="E159" s="5"/>
     </row>
     <row r="160" spans="1:5">
-      <c r="A160" s="5"/>
-      <c r="B160" s="3"/>
-      <c r="C160" s="4"/>
+      <c r="A160" s="2">
+        <v>46270</v>
+      </c>
+      <c r="B160" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C160" s="9">
+        <v>6</v>
+      </c>
       <c r="D160" s="5"/>
       <c r="E160" s="5"/>
     </row>
     <row r="161" spans="1:5">
-      <c r="A161" s="5"/>
-      <c r="B161" s="3"/>
-      <c r="C161" s="4"/>
+      <c r="A161" s="2">
+        <v>46271</v>
+      </c>
+      <c r="B161" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C161" s="9">
+        <v>6</v>
+      </c>
       <c r="D161" s="5"/>
       <c r="E161" s="5"/>
     </row>
     <row r="162" spans="1:5">
-      <c r="A162" s="5"/>
-      <c r="B162" s="3"/>
-      <c r="C162" s="4"/>
+      <c r="A162" s="2">
+        <v>46272</v>
+      </c>
+      <c r="B162" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C162" s="9">
+        <v>6</v>
+      </c>
       <c r="D162" s="5"/>
       <c r="E162" s="5"/>
     </row>
     <row r="163" spans="1:5">
-      <c r="A163" s="5"/>
-      <c r="B163" s="3"/>
-      <c r="C163" s="4"/>
+      <c r="A163" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B163" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C163" s="9">
+        <v>6</v>
+      </c>
       <c r="D163" s="5"/>
       <c r="E163" s="5"/>
     </row>
     <row r="164" spans="1:5">
-      <c r="A164" s="5"/>
-      <c r="B164" s="3"/>
-      <c r="C164" s="4"/>
+      <c r="A164" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B164" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C164" s="9">
+        <v>6</v>
+      </c>
       <c r="D164" s="5"/>
       <c r="E164" s="5"/>
     </row>
     <row r="165" spans="1:5">
-      <c r="A165" s="5"/>
-      <c r="B165" s="3"/>
-      <c r="C165" s="4"/>
+      <c r="A165" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B165" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C165" s="9">
+        <v>6</v>
+      </c>
       <c r="D165" s="5"/>
       <c r="E165" s="5"/>
     </row>
     <row r="166" spans="1:5">
-      <c r="A166" s="5"/>
-      <c r="B166" s="3"/>
-      <c r="C166" s="4"/>
+      <c r="A166" s="2">
+        <v>46276</v>
+      </c>
+      <c r="B166" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C166" s="9">
+        <v>6</v>
+      </c>
       <c r="D166" s="5"/>
       <c r="E166" s="5"/>
     </row>
     <row r="167" spans="1:5">
-      <c r="A167" s="5"/>
-      <c r="B167" s="3"/>
-      <c r="C167" s="4"/>
+      <c r="A167" s="2">
+        <v>46277</v>
+      </c>
+      <c r="B167" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C167" s="9">
+        <v>6</v>
+      </c>
       <c r="D167" s="5"/>
       <c r="E167" s="5"/>
     </row>
     <row r="168" spans="1:5">
-      <c r="A168" s="5"/>
-      <c r="B168" s="3"/>
-      <c r="C168" s="4"/>
+      <c r="A168" s="2">
+        <v>46278</v>
+      </c>
+      <c r="B168" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C168" s="9">
+        <v>6</v>
+      </c>
       <c r="D168" s="5"/>
       <c r="E168" s="5"/>
     </row>
     <row r="169" spans="1:5">
-      <c r="A169" s="5"/>
-      <c r="B169" s="3"/>
-      <c r="C169" s="4"/>
+      <c r="A169" s="2">
+        <v>46279</v>
+      </c>
+      <c r="B169" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C169" s="9">
+        <v>6</v>
+      </c>
       <c r="D169" s="5"/>
       <c r="E169" s="5"/>
     </row>
     <row r="170" spans="1:5">
-      <c r="A170" s="5"/>
-      <c r="B170" s="3"/>
-      <c r="C170" s="4"/>
+      <c r="A170" s="2">
+        <v>46280</v>
+      </c>
+      <c r="B170" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C170" s="9">
+        <v>6</v>
+      </c>
       <c r="D170" s="5"/>
       <c r="E170" s="5"/>
     </row>
     <row r="171" spans="1:5">
-      <c r="A171" s="5"/>
-      <c r="B171" s="3"/>
-      <c r="C171" s="4"/>
+      <c r="A171" s="2">
+        <v>46281</v>
+      </c>
+      <c r="B171" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C171" s="9">
+        <v>6</v>
+      </c>
       <c r="D171" s="5"/>
       <c r="E171" s="5"/>
     </row>
     <row r="172" spans="1:5">
-      <c r="A172" s="5"/>
-      <c r="B172" s="3"/>
-      <c r="C172" s="4"/>
+      <c r="A172" s="2">
+        <v>46282</v>
+      </c>
+      <c r="B172" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C172" s="9">
+        <v>6</v>
+      </c>
       <c r="D172" s="5"/>
       <c r="E172" s="5"/>
     </row>
     <row r="173" spans="1:5">
-      <c r="A173" s="5"/>
-      <c r="B173" s="3"/>
-      <c r="C173" s="4"/>
+      <c r="A173" s="2">
+        <v>46283</v>
+      </c>
+      <c r="B173" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C173" s="9">
+        <v>6</v>
+      </c>
       <c r="D173" s="5"/>
       <c r="E173" s="5"/>
     </row>
     <row r="174" spans="1:5">
-      <c r="A174" s="5"/>
-      <c r="B174" s="3"/>
-      <c r="C174" s="4"/>
+      <c r="A174" s="2">
+        <v>46284</v>
+      </c>
+      <c r="B174" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C174" s="9">
+        <v>6</v>
+      </c>
       <c r="D174" s="5"/>
       <c r="E174" s="5"/>
     </row>
     <row r="175" spans="1:5">
-      <c r="A175" s="5"/>
-      <c r="B175" s="3"/>
-      <c r="C175" s="4"/>
+      <c r="A175" s="2">
+        <v>46285</v>
+      </c>
+      <c r="B175" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C175" s="9">
+        <v>6</v>
+      </c>
       <c r="D175" s="5"/>
       <c r="E175" s="5"/>
     </row>
     <row r="176" spans="1:5">
-      <c r="A176" s="5"/>
-      <c r="B176" s="3"/>
-      <c r="C176" s="4"/>
+      <c r="A176" s="2">
+        <v>46286</v>
+      </c>
+      <c r="B176" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C176" s="9">
+        <v>6</v>
+      </c>
       <c r="D176" s="5"/>
       <c r="E176" s="5"/>
     </row>
     <row r="177" spans="1:5">
-      <c r="A177" s="5"/>
-      <c r="B177" s="3"/>
-      <c r="C177" s="4"/>
+      <c r="A177" s="2">
+        <v>46287</v>
+      </c>
+      <c r="B177" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C177" s="9">
+        <v>6</v>
+      </c>
       <c r="D177" s="5"/>
       <c r="E177" s="5"/>
     </row>
     <row r="178" spans="1:5">
-      <c r="A178" s="5"/>
-      <c r="B178" s="3"/>
-      <c r="C178" s="4"/>
+      <c r="A178" s="2">
+        <v>46288</v>
+      </c>
+      <c r="B178" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C178" s="9">
+        <v>6</v>
+      </c>
       <c r="D178" s="5"/>
       <c r="E178" s="5"/>
     </row>
     <row r="179" spans="1:5">
-      <c r="A179" s="5"/>
-      <c r="B179" s="3"/>
-      <c r="C179" s="4"/>
+      <c r="A179" s="2">
+        <v>46289</v>
+      </c>
+      <c r="B179" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C179" s="9">
+        <v>6</v>
+      </c>
       <c r="D179" s="5"/>
       <c r="E179" s="5"/>
     </row>
     <row r="180" spans="1:5">
-      <c r="A180" s="5"/>
-      <c r="B180" s="3"/>
-      <c r="C180" s="4"/>
+      <c r="A180" s="2">
+        <v>46290</v>
+      </c>
+      <c r="B180" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C180" s="9">
+        <v>6</v>
+      </c>
       <c r="D180" s="5"/>
       <c r="E180" s="5"/>
     </row>
     <row r="181" spans="1:5">
-      <c r="A181" s="5"/>
-      <c r="B181" s="3"/>
-      <c r="C181" s="4"/>
+      <c r="A181" s="2">
+        <v>46291</v>
+      </c>
+      <c r="B181" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C181" s="9">
+        <v>6</v>
+      </c>
       <c r="D181" s="5"/>
       <c r="E181" s="5"/>
     </row>
     <row r="182" spans="1:5">
-      <c r="A182" s="5"/>
-      <c r="B182" s="3"/>
-      <c r="C182" s="4"/>
+      <c r="A182" s="2">
+        <v>46292</v>
+      </c>
+      <c r="B182" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C182" s="9">
+        <v>6</v>
+      </c>
       <c r="D182" s="5"/>
       <c r="E182" s="5"/>
     </row>
     <row r="183" spans="1:5">
-      <c r="A183" s="5"/>
-      <c r="B183" s="3"/>
-      <c r="C183" s="4"/>
+      <c r="A183" s="2">
+        <v>46293</v>
+      </c>
+      <c r="B183" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C183" s="9">
+        <v>6</v>
+      </c>
       <c r="D183" s="5"/>
       <c r="E183" s="5"/>
     </row>
     <row r="184" spans="1:5">
-      <c r="A184" s="5"/>
-      <c r="B184" s="3"/>
-      <c r="C184" s="4"/>
+      <c r="A184" s="2">
+        <v>46294</v>
+      </c>
+      <c r="B184" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C184" s="9">
+        <v>6</v>
+      </c>
       <c r="D184" s="5"/>
       <c r="E184" s="5"/>
     </row>
     <row r="185" spans="1:5">
-      <c r="A185" s="5"/>
-      <c r="B185" s="3"/>
-      <c r="C185" s="4"/>
+      <c r="A185" s="2">
+        <v>46295</v>
+      </c>
+      <c r="B185" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C185" s="9">
+        <v>6</v>
+      </c>
       <c r="D185" s="5"/>
       <c r="E185" s="5"/>
     </row>
     <row r="186" spans="1:5">
-      <c r="A186" s="5"/>
-      <c r="B186" s="3"/>
-      <c r="C186" s="4"/>
+      <c r="A186" s="2">
+        <v>46266</v>
+      </c>
+      <c r="B186" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C186" s="9">
+        <v>9</v>
+      </c>
       <c r="D186" s="5"/>
       <c r="E186" s="5"/>
     </row>
     <row r="187" spans="1:5">
-      <c r="A187" s="5"/>
-      <c r="B187" s="3"/>
-      <c r="C187" s="4"/>
+      <c r="A187" s="2">
+        <v>46267</v>
+      </c>
+      <c r="B187" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C187" s="9">
+        <v>9</v>
+      </c>
       <c r="D187" s="5"/>
       <c r="E187" s="5"/>
     </row>
     <row r="188" spans="1:5">
-      <c r="A188" s="5"/>
-      <c r="B188" s="3"/>
-      <c r="C188" s="4"/>
+      <c r="A188" s="2">
+        <v>46268</v>
+      </c>
+      <c r="B188" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C188" s="9">
+        <v>9</v>
+      </c>
       <c r="D188" s="5"/>
       <c r="E188" s="5"/>
     </row>
     <row r="189" spans="1:5">
-      <c r="A189" s="5"/>
-      <c r="B189" s="3"/>
-      <c r="C189" s="4"/>
+      <c r="A189" s="2">
+        <v>46269</v>
+      </c>
+      <c r="B189" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C189" s="9">
+        <v>9</v>
+      </c>
       <c r="D189" s="5"/>
       <c r="E189" s="5"/>
     </row>
     <row r="190" spans="1:5">
-      <c r="A190" s="5"/>
-      <c r="B190" s="3"/>
-      <c r="C190" s="4"/>
+      <c r="A190" s="2">
+        <v>46270</v>
+      </c>
+      <c r="B190" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C190" s="9">
+        <v>9</v>
+      </c>
       <c r="D190" s="5"/>
       <c r="E190" s="5"/>
     </row>
     <row r="191" spans="1:5">
-      <c r="A191" s="5"/>
-      <c r="B191" s="3"/>
-      <c r="C191" s="4"/>
+      <c r="A191" s="2">
+        <v>46271</v>
+      </c>
+      <c r="B191" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C191" s="9">
+        <v>9</v>
+      </c>
       <c r="D191" s="5"/>
       <c r="E191" s="5"/>
     </row>
     <row r="192" spans="1:5">
-      <c r="A192" s="9"/>
-      <c r="B192" s="3"/>
-      <c r="C192" s="4"/>
-      <c r="D192" s="9"/>
-      <c r="E192" s="9"/>
+      <c r="A192" s="2">
+        <v>46272</v>
+      </c>
+      <c r="B192" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C192" s="9">
+        <v>9</v>
+      </c>
+      <c r="D192" s="10"/>
+      <c r="E192" s="10"/>
     </row>
     <row r="193" spans="1:5">
-      <c r="A193" s="5"/>
-      <c r="B193" s="3"/>
-      <c r="C193" s="4"/>
+      <c r="A193" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B193" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C193" s="9">
+        <v>9</v>
+      </c>
       <c r="D193" s="5"/>
       <c r="E193" s="5"/>
     </row>
     <row r="194" spans="1:5">
-      <c r="A194" s="5"/>
-      <c r="B194" s="3"/>
-      <c r="C194" s="4"/>
+      <c r="A194" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B194" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C194" s="9">
+        <v>9</v>
+      </c>
       <c r="D194" s="5"/>
       <c r="E194" s="5"/>
     </row>
     <row r="195" spans="1:5">
-      <c r="A195" s="5"/>
-      <c r="B195" s="3"/>
-      <c r="C195" s="4"/>
+      <c r="A195" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B195" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C195" s="9">
+        <v>9</v>
+      </c>
       <c r="D195" s="5"/>
       <c r="E195" s="5"/>
     </row>
     <row r="196" spans="1:5">
-      <c r="A196" s="5"/>
-      <c r="B196" s="3"/>
-      <c r="C196" s="4"/>
+      <c r="A196" s="2">
+        <v>46276</v>
+      </c>
+      <c r="B196" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C196" s="9">
+        <v>9</v>
+      </c>
       <c r="D196" s="5"/>
       <c r="E196" s="5"/>
     </row>
     <row r="197" spans="1:5">
-      <c r="A197" s="9"/>
-      <c r="B197" s="3"/>
-      <c r="C197" s="4"/>
-      <c r="D197" s="9"/>
-      <c r="E197" s="9"/>
+      <c r="A197" s="2">
+        <v>46277</v>
+      </c>
+      <c r="B197" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C197" s="9">
+        <v>9</v>
+      </c>
+      <c r="D197" s="10"/>
+      <c r="E197" s="10"/>
     </row>
     <row r="198" spans="1:5">
-      <c r="A198" s="5"/>
-      <c r="B198" s="3"/>
-      <c r="C198" s="4"/>
+      <c r="A198" s="2">
+        <v>46278</v>
+      </c>
+      <c r="B198" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C198" s="9">
+        <v>9</v>
+      </c>
       <c r="D198" s="5"/>
       <c r="E198" s="5"/>
     </row>
     <row r="199" spans="1:5">
-      <c r="A199" s="5"/>
-      <c r="B199" s="3"/>
-      <c r="C199" s="4"/>
+      <c r="A199" s="2">
+        <v>46279</v>
+      </c>
+      <c r="B199" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C199" s="9">
+        <v>9</v>
+      </c>
       <c r="D199" s="5"/>
       <c r="E199" s="5"/>
     </row>
     <row r="200" spans="1:5">
-      <c r="A200" s="5"/>
-      <c r="B200" s="3"/>
-      <c r="C200" s="4"/>
+      <c r="A200" s="2">
+        <v>46280</v>
+      </c>
+      <c r="B200" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C200" s="9">
+        <v>9</v>
+      </c>
       <c r="D200" s="5"/>
       <c r="E200" s="5"/>
     </row>
     <row r="201" spans="1:5">
-      <c r="A201" s="5"/>
-      <c r="B201" s="3"/>
-      <c r="C201" s="4"/>
+      <c r="A201" s="2">
+        <v>46281</v>
+      </c>
+      <c r="B201" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C201" s="9">
+        <v>9</v>
+      </c>
       <c r="D201" s="5"/>
       <c r="E201" s="5"/>
     </row>
     <row r="202" spans="1:5">
-      <c r="A202" s="9"/>
-      <c r="B202" s="3"/>
-      <c r="C202" s="4"/>
-      <c r="D202" s="9"/>
-      <c r="E202" s="9"/>
+      <c r="A202" s="2">
+        <v>46282</v>
+      </c>
+      <c r="B202" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C202" s="9">
+        <v>9</v>
+      </c>
+      <c r="D202" s="10"/>
+      <c r="E202" s="10"/>
     </row>
     <row r="203" spans="1:5">
-      <c r="A203" s="5"/>
-      <c r="B203" s="3"/>
-      <c r="C203" s="4"/>
+      <c r="A203" s="2">
+        <v>46283</v>
+      </c>
+      <c r="B203" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C203" s="9">
+        <v>9</v>
+      </c>
       <c r="D203" s="5"/>
       <c r="E203" s="5"/>
     </row>
     <row r="204" spans="1:5">
-      <c r="A204" s="5"/>
-      <c r="B204" s="3"/>
-      <c r="C204" s="4"/>
+      <c r="A204" s="2">
+        <v>46284</v>
+      </c>
+      <c r="B204" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C204" s="9">
+        <v>9</v>
+      </c>
       <c r="D204" s="5"/>
       <c r="E204" s="5"/>
     </row>
     <row r="205" spans="1:5">
-      <c r="A205" s="5"/>
-      <c r="B205" s="3"/>
-      <c r="C205" s="4"/>
+      <c r="A205" s="2">
+        <v>46285</v>
+      </c>
+      <c r="B205" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C205" s="9">
+        <v>9</v>
+      </c>
       <c r="D205" s="5"/>
       <c r="E205" s="5"/>
     </row>
     <row r="206" spans="1:5">
-      <c r="A206" s="5"/>
-      <c r="B206" s="3"/>
-      <c r="C206" s="4"/>
+      <c r="A206" s="2">
+        <v>46286</v>
+      </c>
+      <c r="B206" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C206" s="9">
+        <v>9</v>
+      </c>
       <c r="D206" s="5"/>
       <c r="E206" s="5"/>
     </row>
     <row r="207" spans="1:5">
-      <c r="A207" s="5"/>
-      <c r="B207" s="3"/>
-      <c r="C207" s="4"/>
+      <c r="A207" s="2">
+        <v>46287</v>
+      </c>
+      <c r="B207" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C207" s="9">
+        <v>9</v>
+      </c>
       <c r="D207" s="5"/>
       <c r="E207" s="5"/>
     </row>
     <row r="208" spans="1:5">
-      <c r="A208" s="9"/>
-      <c r="B208" s="3"/>
-      <c r="C208" s="4"/>
-      <c r="D208" s="9"/>
-      <c r="E208" s="9"/>
+      <c r="A208" s="2">
+        <v>46288</v>
+      </c>
+      <c r="B208" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C208" s="9">
+        <v>9</v>
+      </c>
+      <c r="D208" s="10"/>
+      <c r="E208" s="10"/>
     </row>
     <row r="209" spans="1:5">
-      <c r="A209" s="5"/>
-      <c r="B209" s="3"/>
-      <c r="C209" s="4"/>
+      <c r="A209" s="2">
+        <v>46289</v>
+      </c>
+      <c r="B209" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C209" s="9">
+        <v>9</v>
+      </c>
       <c r="D209" s="5"/>
       <c r="E209" s="5"/>
     </row>
     <row r="210" spans="1:5">
-      <c r="A210" s="5"/>
-      <c r="B210" s="3"/>
-      <c r="C210" s="4"/>
+      <c r="A210" s="2">
+        <v>46290</v>
+      </c>
+      <c r="B210" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C210" s="9">
+        <v>9</v>
+      </c>
       <c r="D210" s="5"/>
       <c r="E210" s="5"/>
     </row>
     <row r="211" spans="1:5">
-      <c r="A211" s="5"/>
-      <c r="B211" s="3"/>
-      <c r="C211" s="4"/>
+      <c r="A211" s="2">
+        <v>46291</v>
+      </c>
+      <c r="B211" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C211" s="9">
+        <v>9</v>
+      </c>
       <c r="D211" s="5"/>
       <c r="E211" s="5"/>
     </row>
     <row r="212" spans="1:5">
-      <c r="A212" s="5"/>
-      <c r="B212" s="3"/>
-      <c r="C212" s="4"/>
+      <c r="A212" s="2">
+        <v>46292</v>
+      </c>
+      <c r="B212" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C212" s="9">
+        <v>9</v>
+      </c>
       <c r="D212" s="5"/>
       <c r="E212" s="5"/>
     </row>
     <row r="213" spans="1:5">
-      <c r="A213" s="5"/>
-      <c r="B213" s="3"/>
-      <c r="C213" s="4"/>
+      <c r="A213" s="2">
+        <v>46293</v>
+      </c>
+      <c r="B213" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C213" s="9">
+        <v>9</v>
+      </c>
       <c r="D213" s="5"/>
       <c r="E213" s="5"/>
     </row>
     <row r="214" spans="1:5">
-      <c r="A214" s="5"/>
-      <c r="B214" s="3"/>
-      <c r="C214" s="4"/>
+      <c r="A214" s="2">
+        <v>46294</v>
+      </c>
+      <c r="B214" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C214" s="9">
+        <v>9</v>
+      </c>
       <c r="D214" s="5"/>
       <c r="E214" s="5"/>
     </row>
     <row r="215" spans="1:5">
-      <c r="A215" s="5"/>
-      <c r="B215" s="3"/>
-      <c r="C215" s="4"/>
+      <c r="A215" s="2">
+        <v>46295</v>
+      </c>
+      <c r="B215" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C215" s="9">
+        <v>9</v>
+      </c>
       <c r="D215" s="5"/>
       <c r="E215" s="5"/>
     </row>
     <row r="216" spans="1:5">
-      <c r="A216" s="5"/>
-      <c r="B216" s="3"/>
-      <c r="C216" s="4"/>
+      <c r="A216" s="2">
+        <v>46266</v>
+      </c>
+      <c r="B216" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C216" s="9">
+        <v>9</v>
+      </c>
       <c r="D216" s="5"/>
       <c r="E216" s="5"/>
     </row>
     <row r="217" spans="1:5">
-      <c r="A217" s="5"/>
-      <c r="B217" s="3"/>
-      <c r="C217" s="4"/>
+      <c r="A217" s="2">
+        <v>46267</v>
+      </c>
+      <c r="B217" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C217" s="9">
+        <v>9</v>
+      </c>
       <c r="D217" s="5"/>
       <c r="E217" s="5"/>
     </row>
     <row r="218" spans="1:5">
-      <c r="A218" s="5"/>
-      <c r="B218" s="3"/>
-      <c r="C218" s="4"/>
+      <c r="A218" s="2">
+        <v>46268</v>
+      </c>
+      <c r="B218" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C218" s="9">
+        <v>9</v>
+      </c>
       <c r="D218" s="5"/>
       <c r="E218" s="5"/>
     </row>
     <row r="219" spans="1:5">
-      <c r="A219" s="5"/>
-      <c r="B219" s="3"/>
-      <c r="C219" s="4"/>
+      <c r="A219" s="2">
+        <v>46269</v>
+      </c>
+      <c r="B219" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C219" s="9">
+        <v>9</v>
+      </c>
       <c r="D219" s="5"/>
       <c r="E219" s="5"/>
     </row>
     <row r="220" spans="1:5">
-      <c r="A220" s="5"/>
-      <c r="B220" s="3"/>
-      <c r="C220" s="4"/>
+      <c r="A220" s="2">
+        <v>46270</v>
+      </c>
+      <c r="B220" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C220" s="9">
+        <v>9</v>
+      </c>
       <c r="D220" s="5"/>
       <c r="E220" s="5"/>
     </row>
     <row r="221" spans="1:5">
-      <c r="A221" s="5"/>
-      <c r="B221" s="3"/>
-      <c r="C221" s="4"/>
+      <c r="A221" s="2">
+        <v>46271</v>
+      </c>
+      <c r="B221" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C221" s="9">
+        <v>9</v>
+      </c>
       <c r="D221" s="5"/>
       <c r="E221" s="5"/>
     </row>
     <row r="222" spans="1:5">
-      <c r="A222" s="5"/>
-      <c r="B222" s="3"/>
-      <c r="C222" s="4"/>
+      <c r="A222" s="2">
+        <v>46272</v>
+      </c>
+      <c r="B222" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C222" s="9">
+        <v>9</v>
+      </c>
       <c r="D222" s="5"/>
       <c r="E222" s="5"/>
     </row>
     <row r="223" spans="1:5">
-      <c r="A223" s="5"/>
-      <c r="B223" s="3"/>
-      <c r="C223" s="4"/>
+      <c r="A223" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B223" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C223" s="9">
+        <v>9</v>
+      </c>
       <c r="D223" s="5"/>
       <c r="E223" s="5"/>
     </row>
     <row r="224" spans="1:5">
-      <c r="A224" s="5"/>
-      <c r="B224" s="3"/>
-      <c r="C224" s="4"/>
+      <c r="A224" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B224" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C224" s="9">
+        <v>9</v>
+      </c>
       <c r="D224" s="5"/>
       <c r="E224" s="5"/>
     </row>
     <row r="225" spans="1:5">
-      <c r="A225" s="5"/>
-      <c r="B225" s="3"/>
-      <c r="C225" s="4"/>
+      <c r="A225" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B225" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C225" s="9">
+        <v>9</v>
+      </c>
       <c r="D225" s="5"/>
       <c r="E225" s="5"/>
     </row>
     <row r="226" spans="1:5">
-      <c r="A226" s="5"/>
-      <c r="B226" s="3"/>
-      <c r="C226" s="4"/>
+      <c r="A226" s="2">
+        <v>46276</v>
+      </c>
+      <c r="B226" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C226" s="9">
+        <v>9</v>
+      </c>
       <c r="D226" s="5"/>
       <c r="E226" s="5"/>
     </row>
     <row r="227" spans="1:5">
-      <c r="A227" s="5"/>
-      <c r="B227" s="3"/>
-      <c r="C227" s="4"/>
+      <c r="A227" s="2">
+        <v>46277</v>
+      </c>
+      <c r="B227" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C227" s="9">
+        <v>9</v>
+      </c>
       <c r="D227" s="5"/>
       <c r="E227" s="5"/>
     </row>
     <row r="228" spans="1:5">
-      <c r="A228" s="3"/>
-      <c r="B228" s="3"/>
-      <c r="C228" s="4"/>
+      <c r="A228" s="2">
+        <v>46278</v>
+      </c>
+      <c r="B228" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C228" s="9">
+        <v>9</v>
+      </c>
       <c r="D228" s="3"/>
       <c r="E228" s="3"/>
     </row>
     <row r="229" spans="1:5">
-      <c r="A229" s="3"/>
-      <c r="B229" s="3"/>
-      <c r="C229" s="4"/>
+      <c r="A229" s="2">
+        <v>46279</v>
+      </c>
+      <c r="B229" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C229" s="9">
+        <v>9</v>
+      </c>
       <c r="D229" s="3"/>
       <c r="E229" s="3"/>
     </row>
     <row r="230" spans="1:5">
-      <c r="A230" s="3"/>
-      <c r="B230" s="3"/>
-      <c r="C230" s="4"/>
+      <c r="A230" s="2">
+        <v>46280</v>
+      </c>
+      <c r="B230" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C230" s="9">
+        <v>9</v>
+      </c>
       <c r="D230" s="3"/>
       <c r="E230" s="3"/>
     </row>
     <row r="231" spans="1:5">
-      <c r="A231" s="3"/>
-      <c r="B231" s="3"/>
-      <c r="C231" s="4"/>
+      <c r="A231" s="2">
+        <v>46281</v>
+      </c>
+      <c r="B231" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C231" s="9">
+        <v>9</v>
+      </c>
       <c r="D231" s="3"/>
       <c r="E231" s="3"/>
     </row>
     <row r="232" spans="1:5">
-      <c r="A232" s="3"/>
-      <c r="B232" s="3"/>
-      <c r="C232" s="4"/>
+      <c r="A232" s="2">
+        <v>46282</v>
+      </c>
+      <c r="B232" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C232" s="9">
+        <v>9</v>
+      </c>
       <c r="D232" s="3"/>
       <c r="E232" s="3"/>
     </row>
+    <row r="233" spans="1:5">
+      <c r="A233" s="2">
+        <v>46283</v>
+      </c>
+      <c r="B233" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C233" s="9">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="234" spans="1:5">
+      <c r="A234" s="2">
+        <v>46284</v>
+      </c>
+      <c r="B234" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C234" s="9">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="235" spans="1:5">
+      <c r="A235" s="2">
+        <v>46285</v>
+      </c>
+      <c r="B235" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C235" s="9">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="236" spans="1:5">
+      <c r="A236" s="2">
+        <v>46286</v>
+      </c>
+      <c r="B236" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C236" s="9">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="237" spans="1:5">
+      <c r="A237" s="2">
+        <v>46287</v>
+      </c>
+      <c r="B237" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C237" s="9">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="238" spans="1:5">
+      <c r="A238" s="2">
+        <v>46288</v>
+      </c>
+      <c r="B238" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C238" s="9">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="239" spans="1:5">
+      <c r="A239" s="2">
+        <v>46289</v>
+      </c>
+      <c r="B239" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C239" s="9">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="240" spans="1:5">
+      <c r="A240" s="2">
+        <v>46290</v>
+      </c>
+      <c r="B240" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C240" s="9">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="241" spans="1:3">
+      <c r="A241" s="2">
+        <v>46291</v>
+      </c>
+      <c r="B241" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C241" s="9">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="242" spans="1:3">
+      <c r="A242" s="2">
+        <v>46292</v>
+      </c>
+      <c r="B242" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C242" s="9">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="243" spans="1:3">
+      <c r="A243" s="2">
+        <v>46293</v>
+      </c>
+      <c r="B243" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C243" s="9">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="244" spans="1:3">
+      <c r="A244" s="2">
+        <v>46294</v>
+      </c>
+      <c r="B244" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C244" s="9">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="245" spans="1:3">
+      <c r="A245" s="2">
+        <v>46295</v>
+      </c>
+      <c r="B245" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C245" s="9">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="246" spans="1:3">
+      <c r="A246" s="2">
+        <v>46266</v>
+      </c>
+      <c r="B246" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C246" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="247" spans="1:3">
+      <c r="A247" s="2">
+        <v>46267</v>
+      </c>
+      <c r="B247" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C247" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="248" spans="1:3">
+      <c r="A248" s="2">
+        <v>46268</v>
+      </c>
+      <c r="B248" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C248" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="249" spans="1:3">
+      <c r="A249" s="2">
+        <v>46269</v>
+      </c>
+      <c r="B249" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C249" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="250" spans="1:3">
+      <c r="A250" s="2">
+        <v>46270</v>
+      </c>
+      <c r="B250" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C250" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="251" spans="1:3">
+      <c r="A251" s="2">
+        <v>46271</v>
+      </c>
+      <c r="B251" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C251" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="252" spans="1:3">
+      <c r="A252" s="2">
+        <v>46272</v>
+      </c>
+      <c r="B252" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C252" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="253" spans="1:3">
+      <c r="A253" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B253" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C253" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="254" spans="1:3">
+      <c r="A254" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B254" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C254" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="255" spans="1:3">
+      <c r="A255" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B255" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C255" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="256" spans="1:3">
+      <c r="A256" s="2">
+        <v>46276</v>
+      </c>
+      <c r="B256" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C256" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="257" spans="1:3">
+      <c r="A257" s="2">
+        <v>46277</v>
+      </c>
+      <c r="B257" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C257" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="258" spans="1:3">
+      <c r="A258" s="2">
+        <v>46278</v>
+      </c>
+      <c r="B258" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C258" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="259" spans="1:3">
+      <c r="A259" s="2">
+        <v>46279</v>
+      </c>
+      <c r="B259" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C259" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="260" spans="1:3">
+      <c r="A260" s="2">
+        <v>46280</v>
+      </c>
+      <c r="B260" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C260" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="261" spans="1:3">
+      <c r="A261" s="2">
+        <v>46281</v>
+      </c>
+      <c r="B261" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C261" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="262" spans="1:3">
+      <c r="A262" s="2">
+        <v>46282</v>
+      </c>
+      <c r="B262" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C262" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="263" spans="1:3">
+      <c r="A263" s="2">
+        <v>46283</v>
+      </c>
+      <c r="B263" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C263" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="264" spans="1:3">
+      <c r="A264" s="2">
+        <v>46284</v>
+      </c>
+      <c r="B264" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C264" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="265" spans="1:3">
+      <c r="A265" s="2">
+        <v>46285</v>
+      </c>
+      <c r="B265" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C265" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="266" spans="1:3">
+      <c r="A266" s="2">
+        <v>46286</v>
+      </c>
+      <c r="B266" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C266" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="267" spans="1:3">
+      <c r="A267" s="2">
+        <v>46287</v>
+      </c>
+      <c r="B267" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C267" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="268" spans="1:3">
+      <c r="A268" s="2">
+        <v>46288</v>
+      </c>
+      <c r="B268" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C268" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="269" spans="1:3">
+      <c r="A269" s="2">
+        <v>46289</v>
+      </c>
+      <c r="B269" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C269" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="270" spans="1:3">
+      <c r="A270" s="2">
+        <v>46290</v>
+      </c>
+      <c r="B270" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C270" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="271" spans="1:3">
+      <c r="A271" s="2">
+        <v>46291</v>
+      </c>
+      <c r="B271" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C271" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="272" spans="1:3">
+      <c r="A272" s="2">
+        <v>46292</v>
+      </c>
+      <c r="B272" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C272" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="273" spans="1:3">
+      <c r="A273" s="2">
+        <v>46293</v>
+      </c>
+      <c r="B273" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C273" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="274" spans="1:3">
+      <c r="A274" s="2">
+        <v>46294</v>
+      </c>
+      <c r="B274" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C274" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="275" spans="1:3">
+      <c r="A275" s="2">
+        <v>46295</v>
+      </c>
+      <c r="B275" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C275" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="276" spans="1:3">
+      <c r="B276" s="3"/>
+    </row>
+    <row r="277" spans="1:3">
+      <c r="B277" s="3"/>
+    </row>
   </sheetData>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:T232" etc:filterBottomFollowUsedRange="0">
-    <sortState ref="A2:T232">
+    <sortState ref="A1:T232">
       <sortCondition ref="A1"/>
     </sortState>
     <extLst/>

</xml_diff>